<commit_message>
Enhance Likert Engine: Add normalization and conversion functions for improved value handling
</commit_message>
<xml_diff>
--- a/excel/ΣΑΠ-ΦΘ_MASTER.xlsx
+++ b/excel/ΣΑΠ-ΦΘ_MASTER.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,7 +442,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3.16</v>
+        <v>2.98</v>
       </c>
     </row>
     <row r="6">
@@ -455,30 +455,90 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Β</t>
+          <t>Α</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3.33</v>
+        <v>2.83</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Γ</t>
+          <t>Β</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Γ</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Δ</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>Ε</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B12" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Ζ</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Η</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Θ</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ΣΤ</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Add validation report and complete Likert mapping
</commit_message>
<xml_diff>
--- a/excel/ΣΑΠ-ΦΘ_MASTER.xlsx
+++ b/excel/ΣΑΠ-ΦΘ_MASTER.xlsx
@@ -442,7 +442,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2.94</v>
+        <v>2.98</v>
       </c>
     </row>
     <row r="6">
@@ -479,7 +479,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2.93</v>
+        <v>3.23</v>
       </c>
     </row>
     <row r="11">

</xml_diff>